<commit_message>
Actualiza Resumen y despliegue de reporte
- Elimina embudo de la pestaña Resumen.
- Unifica estructura y anchos de filas/columnas en Resumen.
- Corrige Año anterior y % vs año anterior con período YoY equivalente.
- Incluye actualización del reporte mensual.

Co-Authored-By: Oz <oz-agent@warp.dev>
</commit_message>
<xml_diff>
--- a/reporter/Mosca | Performance | Reporte mensual 2026-04.xlsx
+++ b/reporter/Mosca | Performance | Reporte mensual 2026-04.xlsx
@@ -12,6 +12,7 @@
     <sheet name="Google Ads" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="09-04-2026" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="12-04-2026" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="17-04-2026" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -162,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1"/>
@@ -269,6 +270,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -586,6 +608,390 @@
           <val>
             <numRef>
               <f>'12-04-2026'!$AA$25:$AA$26</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Inversión</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'17-04-2026'!AA4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dLbls>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="1"/>
+            <showSerName val="0"/>
+            <showPercent val="1"/>
+          </dLbls>
+          <cat>
+            <numRef>
+              <f>'17-04-2026'!$Z$5:$Z$6</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'17-04-2026'!$AA$5:$AA$6</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Impresiones</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'17-04-2026'!AA8</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dLbls>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="1"/>
+            <showSerName val="0"/>
+            <showPercent val="1"/>
+          </dLbls>
+          <cat>
+            <numRef>
+              <f>'17-04-2026'!$Z$9:$Z$10</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'17-04-2026'!$AA$9:$AA$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Clicks</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'17-04-2026'!AA12</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dLbls>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="1"/>
+            <showSerName val="0"/>
+            <showPercent val="1"/>
+          </dLbls>
+          <cat>
+            <numRef>
+              <f>'17-04-2026'!$Z$13:$Z$14</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'17-04-2026'!$AA$13:$AA$14</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Sesiones</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'17-04-2026'!AA16</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dLbls>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="1"/>
+            <showSerName val="0"/>
+            <showPercent val="1"/>
+          </dLbls>
+          <cat>
+            <numRef>
+              <f>'17-04-2026'!$Z$17:$Z$18</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'17-04-2026'!$AA$17:$AA$18</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Compras</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'17-04-2026'!AA20</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dLbls>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="1"/>
+            <showSerName val="0"/>
+            <showPercent val="1"/>
+          </dLbls>
+          <cat>
+            <numRef>
+              <f>'17-04-2026'!$Z$21:$Z$22</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'17-04-2026'!$AA$21:$AA$22</f>
+            </numRef>
+          </val>
+        </ser>
+        <firstSliceAng val="0"/>
+      </pieChart>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Ingresos</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <pieChart>
+        <varyColors val="1"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'17-04-2026'!AA24</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <dLbls>
+            <showLegendKey val="0"/>
+            <showVal val="0"/>
+            <showCatName val="1"/>
+            <showSerName val="0"/>
+            <showPercent val="1"/>
+          </dLbls>
+          <cat>
+            <numRef>
+              <f>'17-04-2026'!$Z$25:$Z$26</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'17-04-2026'!$AA$25:$AA$26</f>
             </numRef>
           </val>
         </ser>
@@ -1542,6 +1948,171 @@
 </wsDr>
 </file>
 
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>31</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2880000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>38</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2880000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>46</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2880000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>31</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2880000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>38</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2880000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="5" name="Chart 5"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>46</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="2880000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="6" name="Chart 6"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId6"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>0</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="419100" cy="419100"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1831,10 +2402,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V19"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
@@ -1857,19 +2428,14 @@
     <col width="6" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="48" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">MOSCA HNOS.  </t>
         </is>
       </c>
-      <c r="K1" s="37" t="inlineStr">
-        <is>
-          <t>EMBUDO DE CONVERSIÓN</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="5" customHeight="1">
+    </row>
+    <row r="2" ht="6" customHeight="1">
       <c r="A2" s="2" t="n"/>
       <c r="B2" s="2" t="n"/>
       <c r="C2" s="2" t="n"/>
@@ -1879,20 +2445,8 @@
       <c r="G2" s="2" t="n"/>
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="n"/>
-      <c r="K2" s="38" t="n"/>
-      <c r="L2" s="38" t="n"/>
-      <c r="M2" s="38" t="n"/>
-      <c r="N2" s="38" t="n"/>
-      <c r="O2" s="38" t="n"/>
-      <c r="P2" s="38" t="n"/>
-      <c r="Q2" s="38" t="n"/>
-      <c r="R2" s="38" t="n"/>
-      <c r="S2" s="38" t="n"/>
-      <c r="T2" s="38" t="n"/>
-      <c r="U2" s="38" t="n"/>
-      <c r="V2" s="38" t="n"/>
-    </row>
-    <row r="3" ht="30" customHeight="1">
+    </row>
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Fecha</t>
@@ -1938,127 +2492,91 @@
           <t>Conv %</t>
         </is>
       </c>
-      <c r="K3" s="39" t="inlineStr">
-        <is>
-          <t>Sesiones   87,891   (100.0%)</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="10" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="48" t="inlineStr">
         <is>
           <t>Año anterior</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>85519</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>4987</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>1670</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>235</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>3905.57</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>11869.348219</v>
-      </c>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="6" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="K4" s="40" t="n"/>
-      <c r="L4" s="41" t="n"/>
-      <c r="M4" s="41" t="n"/>
-      <c r="N4" s="41" t="n"/>
-      <c r="O4" s="41" t="n"/>
-      <c r="P4" s="41" t="n"/>
-      <c r="Q4" s="41" t="n"/>
-      <c r="R4" s="41" t="n"/>
-      <c r="S4" s="41" t="n"/>
-      <c r="T4" s="41" t="n"/>
-      <c r="U4" s="41" t="n"/>
-      <c r="V4" s="40" t="n"/>
+      <c r="B4" s="49" t="n">
+        <v>112895</v>
+      </c>
+      <c r="C4" s="49" t="n">
+        <v>6182</v>
+      </c>
+      <c r="D4" s="49" t="n">
+        <v>2093</v>
+      </c>
+      <c r="E4" s="49" t="n">
+        <v>290</v>
+      </c>
+      <c r="F4" s="50" t="n">
+        <v>5374.43</v>
+      </c>
+      <c r="G4" s="50" t="n">
+        <v>15004.8352</v>
+      </c>
+      <c r="H4" s="49" t="n"/>
+      <c r="I4" s="51" t="n">
+        <v>0.26</v>
+      </c>
     </row>
     <row r="5" ht="4" customHeight="1">
-      <c r="A5" s="7" t="n"/>
-      <c r="B5" s="7" t="n">
-        <v>87891</v>
-      </c>
-      <c r="C5" s="7" t="n">
-        <v>4785</v>
-      </c>
-      <c r="D5" s="7" t="n">
-        <v>2027</v>
-      </c>
-      <c r="E5" s="7" t="n">
-        <v>289</v>
-      </c>
-      <c r="F5" s="8" t="n">
-        <v>4138.19</v>
-      </c>
-      <c r="G5" s="8" t="n">
-        <v>14789.652346</v>
-      </c>
-      <c r="H5" s="7" t="n">
-        <v>3.57</v>
-      </c>
-      <c r="I5" s="9" t="n">
+      <c r="A5" s="14" t="n"/>
+      <c r="B5" s="16" t="n">
+        <v>108662</v>
+      </c>
+      <c r="C5" s="16" t="n">
+        <v>5814</v>
+      </c>
+      <c r="D5" s="16" t="n">
+        <v>2453</v>
+      </c>
+      <c r="E5" s="16" t="n">
+        <v>354</v>
+      </c>
+      <c r="F5" s="15" t="n">
+        <v>4901.079999999999</v>
+      </c>
+      <c r="G5" s="15" t="n">
+        <v>18597.882743</v>
+      </c>
+      <c r="H5" s="16" t="n">
+        <v>3.79</v>
+      </c>
+      <c r="I5" s="17" t="n">
         <v>0.33</v>
       </c>
-      <c r="K5" s="40" t="n"/>
-      <c r="L5" s="40" t="n"/>
-      <c r="M5" s="40" t="n"/>
-      <c r="N5" s="40" t="n"/>
-      <c r="O5" s="40" t="n"/>
-      <c r="P5" s="40" t="n"/>
-      <c r="Q5" s="40" t="n"/>
-      <c r="R5" s="40" t="n"/>
-      <c r="S5" s="40" t="n"/>
-      <c r="T5" s="40" t="n"/>
-      <c r="U5" s="40" t="n"/>
-      <c r="V5" s="40" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="52" t="inlineStr">
         <is>
           <t>% vs año anterior</t>
         </is>
       </c>
-      <c r="B6" s="11" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>-4.1</v>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>23</v>
-      </c>
-      <c r="F6" s="11" t="n">
-        <v>6</v>
-      </c>
-      <c r="G6" s="10" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="11" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="K6" s="40" t="n"/>
-      <c r="L6" s="42" t="inlineStr">
-        <is>
-          <t>Add to Cart   4,785   (5.4%)</t>
-        </is>
-      </c>
-      <c r="V6" s="40" t="n"/>
+      <c r="B6" s="53" t="n">
+        <v>-3.7</v>
+      </c>
+      <c r="C6" s="53" t="n">
+        <v>-6</v>
+      </c>
+      <c r="D6" s="53" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="E6" s="53" t="n">
+        <v>22.1</v>
+      </c>
+      <c r="F6" s="53" t="n">
+        <v>-8.800000000000001</v>
+      </c>
+      <c r="G6" s="54" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="H6" s="54" t="n"/>
+      <c r="I6" s="53" t="n">
+        <v>26.9</v>
+      </c>
     </row>
     <row r="7" ht="10" customHeight="1">
       <c r="A7" t="inlineStr">
@@ -2090,18 +2608,6 @@
       <c r="I7" s="13" t="n">
         <v>0.23</v>
       </c>
-      <c r="K7" s="40" t="n"/>
-      <c r="L7" s="40" t="n"/>
-      <c r="M7" s="43" t="n"/>
-      <c r="N7" s="43" t="n"/>
-      <c r="O7" s="43" t="n"/>
-      <c r="P7" s="43" t="n"/>
-      <c r="Q7" s="43" t="n"/>
-      <c r="R7" s="43" t="n"/>
-      <c r="S7" s="43" t="n"/>
-      <c r="T7" s="43" t="n"/>
-      <c r="U7" s="40" t="n"/>
-      <c r="V7" s="40" t="n"/>
     </row>
     <row r="8" ht="4" customHeight="1">
       <c r="A8" t="inlineStr">
@@ -2133,18 +2639,6 @@
       <c r="I8" s="13" t="n">
         <v>0.15</v>
       </c>
-      <c r="K8" s="40" t="n"/>
-      <c r="L8" s="40" t="n"/>
-      <c r="M8" s="40" t="n"/>
-      <c r="N8" s="40" t="n"/>
-      <c r="O8" s="40" t="n"/>
-      <c r="P8" s="40" t="n"/>
-      <c r="Q8" s="40" t="n"/>
-      <c r="R8" s="40" t="n"/>
-      <c r="S8" s="40" t="n"/>
-      <c r="T8" s="40" t="n"/>
-      <c r="U8" s="40" t="n"/>
-      <c r="V8" s="40" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" t="inlineStr">
@@ -2176,15 +2670,6 @@
       <c r="I9" s="13" t="n">
         <v>0.26</v>
       </c>
-      <c r="K9" s="40" t="n"/>
-      <c r="L9" s="40" t="n"/>
-      <c r="M9" s="44" t="inlineStr">
-        <is>
-          <t>Checkout   2,027   (2.3%)</t>
-        </is>
-      </c>
-      <c r="U9" s="40" t="n"/>
-      <c r="V9" s="40" t="n"/>
     </row>
     <row r="10" ht="10" customHeight="1">
       <c r="A10" t="inlineStr">
@@ -2216,18 +2701,6 @@
       <c r="I10" s="13" t="n">
         <v>0.36</v>
       </c>
-      <c r="K10" s="40" t="n"/>
-      <c r="L10" s="40" t="n"/>
-      <c r="M10" s="40" t="n"/>
-      <c r="N10" s="45" t="n"/>
-      <c r="O10" s="45" t="n"/>
-      <c r="P10" s="45" t="n"/>
-      <c r="Q10" s="45" t="n"/>
-      <c r="R10" s="45" t="n"/>
-      <c r="S10" s="45" t="n"/>
-      <c r="T10" s="40" t="n"/>
-      <c r="U10" s="40" t="n"/>
-      <c r="V10" s="40" t="n"/>
     </row>
     <row r="11" ht="4" customHeight="1">
       <c r="A11" t="inlineStr">
@@ -2259,18 +2732,6 @@
       <c r="I11" s="13" t="n">
         <v>0.39</v>
       </c>
-      <c r="K11" s="40" t="n"/>
-      <c r="L11" s="40" t="n"/>
-      <c r="M11" s="40" t="n"/>
-      <c r="N11" s="40" t="n"/>
-      <c r="O11" s="40" t="n"/>
-      <c r="P11" s="40" t="n"/>
-      <c r="Q11" s="40" t="n"/>
-      <c r="R11" s="40" t="n"/>
-      <c r="S11" s="40" t="n"/>
-      <c r="T11" s="40" t="n"/>
-      <c r="U11" s="40" t="n"/>
-      <c r="V11" s="40" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" t="inlineStr">
@@ -2302,17 +2763,6 @@
       <c r="I12" s="13" t="n">
         <v>0.49</v>
       </c>
-      <c r="K12" s="40" t="n"/>
-      <c r="L12" s="40" t="n"/>
-      <c r="M12" s="40" t="n"/>
-      <c r="N12" s="46" t="inlineStr">
-        <is>
-          <t>Compras   289   (0.3%)</t>
-        </is>
-      </c>
-      <c r="T12" s="40" t="n"/>
-      <c r="U12" s="40" t="n"/>
-      <c r="V12" s="40" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2344,18 +2794,6 @@
       <c r="I13" s="13" t="n">
         <v>0.38</v>
       </c>
-      <c r="K13" s="47" t="n"/>
-      <c r="L13" s="47" t="n"/>
-      <c r="M13" s="47" t="n"/>
-      <c r="N13" s="47" t="n"/>
-      <c r="O13" s="47" t="n"/>
-      <c r="P13" s="47" t="n"/>
-      <c r="Q13" s="47" t="n"/>
-      <c r="R13" s="47" t="n"/>
-      <c r="S13" s="47" t="n"/>
-      <c r="T13" s="47" t="n"/>
-      <c r="U13" s="47" t="n"/>
-      <c r="V13" s="47" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2387,18 +2825,6 @@
       <c r="I14" s="13" t="n">
         <v>0.34</v>
       </c>
-      <c r="K14" s="47" t="n"/>
-      <c r="L14" s="47" t="n"/>
-      <c r="M14" s="47" t="n"/>
-      <c r="N14" s="47" t="n"/>
-      <c r="O14" s="47" t="n"/>
-      <c r="P14" s="47" t="n"/>
-      <c r="Q14" s="47" t="n"/>
-      <c r="R14" s="47" t="n"/>
-      <c r="S14" s="47" t="n"/>
-      <c r="T14" s="47" t="n"/>
-      <c r="U14" s="47" t="n"/>
-      <c r="V14" s="47" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2555,14 +2981,102 @@
         <v>0.41</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>6655</v>
+      </c>
+      <c r="C20" t="n">
+        <v>318</v>
+      </c>
+      <c r="D20" t="n">
+        <v>181</v>
+      </c>
+      <c r="E20" t="n">
+        <v>21</v>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>243.34</v>
+      </c>
+      <c r="G20" s="12" t="n">
+        <v>936.6211179999999</v>
+      </c>
+      <c r="H20" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="I20" s="13" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>6624</v>
+      </c>
+      <c r="C21" t="n">
+        <v>333</v>
+      </c>
+      <c r="D21" t="n">
+        <v>117</v>
+      </c>
+      <c r="E21" t="n">
+        <v>21</v>
+      </c>
+      <c r="F21" s="12" t="n">
+        <v>264.61</v>
+      </c>
+      <c r="G21" s="12" t="n">
+        <v>1769.835326</v>
+      </c>
+      <c r="H21" t="n">
+        <v>6.69</v>
+      </c>
+      <c r="I21" s="13" t="n">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>7492</v>
+      </c>
+      <c r="C22" t="n">
+        <v>378</v>
+      </c>
+      <c r="D22" t="n">
+        <v>128</v>
+      </c>
+      <c r="E22" t="n">
+        <v>23</v>
+      </c>
+      <c r="F22" s="12" t="n">
+        <v>254.49</v>
+      </c>
+      <c r="G22" s="12" t="n">
+        <v>1101.773953</v>
+      </c>
+      <c r="H22" t="n">
+        <v>4.33</v>
+      </c>
+      <c r="I22" s="13" t="n">
+        <v>0.31</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="K1:V1"/>
+  <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="L6:U6"/>
-    <mergeCell ref="M9:T9"/>
-    <mergeCell ref="K3:V3"/>
-    <mergeCell ref="N12:S12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2575,7 +3089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:S20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2594,6 +3108,9 @@
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="14" customWidth="1" min="15" max="15"/>
     <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="48" customHeight="1">
@@ -2620,6 +3137,9 @@
       <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
@@ -2669,35 +3189,50 @@
       </c>
       <c r="J3" s="3" t="inlineStr">
         <is>
+          <t>Compras Meta</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>CPA Meta</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Valor Meta</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
           <t>Sesiones</t>
         </is>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>Add Cart</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="O3" s="3" t="inlineStr">
         <is>
           <t>Checkout</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>Compras</t>
-        </is>
-      </c>
-      <c r="N3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>Compras GA4</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>Ingresos</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t>ROAS</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t>Conv %</t>
         </is>
@@ -2706,53 +3241,62 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>2026-04-01 → 2026-04-13</t>
+          <t>2026-04-01 → 2026-04-16</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>1625.37</v>
+        <v>1906.71</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>1876480</v>
+        <v>2307936</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>2436533</v>
+        <v>2919715</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>0.67</v>
+        <v>0.65</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="G4" s="7" t="n">
-        <v>48649</v>
+        <v>54580</v>
       </c>
       <c r="H4" s="8" t="n">
         <v>0.03</v>
       </c>
       <c r="I4" s="9" t="n">
-        <v>2</v>
+        <v>1.87</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>10344</v>
-      </c>
-      <c r="K4" s="7" t="n">
-        <v>272</v>
-      </c>
-      <c r="L4" s="7" t="n">
-        <v>83</v>
+        <v>333</v>
+      </c>
+      <c r="K4" s="8" t="n">
+        <v>5.73</v>
+      </c>
+      <c r="L4" s="8" t="n">
+        <v>529.04</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="N4" s="8" t="n">
-        <v>367.988186</v>
+        <v>12351</v>
+      </c>
+      <c r="N4" s="7" t="n">
+        <v>336</v>
       </c>
       <c r="O4" s="7" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="P4" s="9" t="n">
-        <v>0.09</v>
+        <v>97</v>
+      </c>
+      <c r="P4" s="7" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q4" s="8" t="n">
+        <v>387.477996</v>
+      </c>
+      <c r="R4" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="S4" s="9" t="n">
+        <v>0.08</v>
       </c>
     </row>
     <row r="5">
@@ -2785,8 +3329,15 @@
       <c r="I5" s="13" t="n">
         <v>1.92</v>
       </c>
-      <c r="N5" s="12" t="n"/>
-      <c r="P5" s="13" t="n"/>
+      <c r="J5" t="n">
+        <v>9</v>
+      </c>
+      <c r="K5" s="12" t="n">
+        <v>13.38</v>
+      </c>
+      <c r="L5" s="12" t="n"/>
+      <c r="Q5" s="12" t="n"/>
+      <c r="S5" s="13" t="n"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2818,8 +3369,17 @@
       <c r="I6" s="13" t="n">
         <v>1.52</v>
       </c>
-      <c r="N6" s="12" t="n"/>
-      <c r="P6" s="13" t="n"/>
+      <c r="J6" t="n">
+        <v>10</v>
+      </c>
+      <c r="K6" s="12" t="n">
+        <v>14.36</v>
+      </c>
+      <c r="L6" s="12" t="n">
+        <v>94.89</v>
+      </c>
+      <c r="Q6" s="12" t="n"/>
+      <c r="S6" s="13" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2851,8 +3411,15 @@
       <c r="I7" s="13" t="n">
         <v>1.48</v>
       </c>
-      <c r="N7" s="12" t="n"/>
-      <c r="P7" s="13" t="n"/>
+      <c r="J7" t="n">
+        <v>17</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="L7" s="12" t="n"/>
+      <c r="Q7" s="12" t="n"/>
+      <c r="S7" s="13" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2884,276 +3451,497 @@
       <c r="I8" s="13" t="n">
         <v>1.42</v>
       </c>
-      <c r="N8" s="12" t="n"/>
-      <c r="P8" s="13" t="n"/>
+      <c r="J8" t="n">
+        <v>11</v>
+      </c>
+      <c r="K8" s="12" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L8" s="12" t="n"/>
+      <c r="Q8" s="12" t="n"/>
+      <c r="S8" s="13" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-04-06</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>152.23</v>
-      </c>
-      <c r="C9" t="n">
-        <v>165620</v>
-      </c>
-      <c r="D9" t="n">
-        <v>218585</v>
-      </c>
-      <c r="E9" s="12" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="F9" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="G9" t="n">
-        <v>4674</v>
-      </c>
-      <c r="H9" s="12" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="I9" s="13" t="n">
-        <v>2.14</v>
-      </c>
-      <c r="N9" s="12" t="n"/>
-      <c r="P9" s="13" t="n"/>
+        <v>0</v>
+      </c>
+      <c r="E9" s="12" t="n"/>
+      <c r="H9" s="12" t="n"/>
+      <c r="I9" s="13" t="n"/>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="12" t="n"/>
+      <c r="Q9" s="12" t="n"/>
+      <c r="S9" s="13" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-06</t>
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>207.7</v>
+        <v>152.23</v>
       </c>
       <c r="C10" t="n">
-        <v>196964</v>
+        <v>165620</v>
       </c>
       <c r="D10" t="n">
-        <v>279380</v>
+        <v>218585</v>
       </c>
       <c r="E10" s="12" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="F10" t="n">
-        <v>1.42</v>
+        <v>1.32</v>
       </c>
       <c r="G10" t="n">
-        <v>6888</v>
+        <v>4674</v>
       </c>
       <c r="H10" s="12" t="n">
         <v>0.03</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>2.47</v>
-      </c>
-      <c r="N10" s="12" t="n"/>
-      <c r="P10" s="13" t="n"/>
+        <v>2.14</v>
+      </c>
+      <c r="J10" t="n">
+        <v>32</v>
+      </c>
+      <c r="K10" s="12" t="n">
+        <v>4.76</v>
+      </c>
+      <c r="L10" s="12" t="n">
+        <v>54.89</v>
+      </c>
+      <c r="Q10" s="12" t="n"/>
+      <c r="S10" s="13" t="n"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-04-08</t>
+          <t>2026-04-07</t>
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>157.08</v>
+        <v>207.7</v>
       </c>
       <c r="C11" t="n">
-        <v>171143</v>
+        <v>196964</v>
       </c>
       <c r="D11" t="n">
-        <v>225899</v>
+        <v>279380</v>
       </c>
       <c r="E11" s="12" t="n">
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
       <c r="F11" t="n">
-        <v>1.32</v>
+        <v>1.42</v>
       </c>
       <c r="G11" t="n">
-        <v>5172</v>
+        <v>6888</v>
       </c>
       <c r="H11" s="12" t="n">
         <v>0.03</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>2.29</v>
-      </c>
-      <c r="N11" s="12" t="n"/>
-      <c r="P11" s="13" t="n"/>
+        <v>2.47</v>
+      </c>
+      <c r="J11" t="n">
+        <v>54</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <v>3.85</v>
+      </c>
+      <c r="L11" s="12" t="n">
+        <v>23.67</v>
+      </c>
+      <c r="Q11" s="12" t="n"/>
+      <c r="S11" s="13" t="n"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-04-09</t>
+          <t>2026-04-08</t>
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>180.09</v>
+        <v>157.08</v>
       </c>
       <c r="C12" t="n">
-        <v>172367</v>
+        <v>171143</v>
       </c>
       <c r="D12" t="n">
-        <v>239014</v>
+        <v>225899</v>
       </c>
       <c r="E12" s="12" t="n">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="F12" t="n">
-        <v>1.39</v>
+        <v>1.32</v>
       </c>
       <c r="G12" t="n">
-        <v>5935</v>
+        <v>5172</v>
       </c>
       <c r="H12" s="12" t="n">
         <v>0.03</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>2.48</v>
-      </c>
-      <c r="N12" s="12" t="n"/>
-      <c r="P12" s="13" t="n"/>
+        <v>2.29</v>
+      </c>
+      <c r="J12" t="n">
+        <v>29</v>
+      </c>
+      <c r="K12" s="12" t="n">
+        <v>5.42</v>
+      </c>
+      <c r="L12" s="12" t="n"/>
+      <c r="Q12" s="12" t="n"/>
+      <c r="S12" s="13" t="n"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>133.54</v>
+        <v>180.09</v>
       </c>
       <c r="C13" t="n">
-        <v>144220</v>
+        <v>172367</v>
       </c>
       <c r="D13" t="n">
-        <v>178416</v>
+        <v>239014</v>
       </c>
       <c r="E13" s="12" t="n">
         <v>0.75</v>
       </c>
       <c r="F13" t="n">
-        <v>1.24</v>
+        <v>1.39</v>
       </c>
       <c r="G13" t="n">
-        <v>4131</v>
+        <v>5935</v>
       </c>
       <c r="H13" s="12" t="n">
         <v>0.03</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>2.32</v>
-      </c>
-      <c r="N13" s="12" t="n"/>
-      <c r="P13" s="13" t="n"/>
+        <v>2.48</v>
+      </c>
+      <c r="J13" t="n">
+        <v>23</v>
+      </c>
+      <c r="K13" s="12" t="n">
+        <v>7.83</v>
+      </c>
+      <c r="L13" s="12" t="n">
+        <v>67.22</v>
+      </c>
+      <c r="Q13" s="12" t="n"/>
+      <c r="S13" s="13" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-04-11</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>113.1</v>
+        <v>133.73</v>
       </c>
       <c r="C14" t="n">
-        <v>133860</v>
+        <v>144573</v>
       </c>
       <c r="D14" t="n">
-        <v>162493</v>
+        <v>178692</v>
       </c>
       <c r="E14" s="12" t="n">
-        <v>0.7</v>
+        <v>0.75</v>
       </c>
       <c r="F14" t="n">
-        <v>1.21</v>
+        <v>1.24</v>
       </c>
       <c r="G14" t="n">
-        <v>2768</v>
+        <v>4138</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="N14" s="12" t="n"/>
-      <c r="P14" s="13" t="n"/>
+        <v>2.32</v>
+      </c>
+      <c r="J14" t="n">
+        <v>25</v>
+      </c>
+      <c r="K14" s="12" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>27.01</v>
+      </c>
+      <c r="Q14" s="12" t="n"/>
+      <c r="S14" s="13" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-04-12</t>
+          <t>2026-04-11</t>
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>144.74</v>
+        <v>113.1</v>
       </c>
       <c r="C15" t="n">
-        <v>163672</v>
+        <v>133860</v>
       </c>
       <c r="D15" t="n">
-        <v>211343</v>
+        <v>162493</v>
       </c>
       <c r="E15" s="12" t="n">
-        <v>0.68</v>
+        <v>0.7</v>
       </c>
       <c r="F15" t="n">
-        <v>1.29</v>
+        <v>1.21</v>
       </c>
       <c r="G15" t="n">
-        <v>4094</v>
+        <v>2768</v>
       </c>
       <c r="H15" s="12" t="n">
         <v>0.04</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>1.94</v>
-      </c>
-      <c r="N15" s="12" t="n"/>
-      <c r="P15" s="13" t="n"/>
+        <v>1.7</v>
+      </c>
+      <c r="J15" t="n">
+        <v>16</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <v>7.07</v>
+      </c>
+      <c r="L15" s="12" t="n"/>
+      <c r="Q15" s="12" t="n"/>
+      <c r="S15" s="13" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-04-13</t>
+          <t>2026-04-12</t>
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>127.23</v>
+        <v>145.34</v>
       </c>
       <c r="C16" t="n">
-        <v>153849</v>
+        <v>163900</v>
       </c>
       <c r="D16" t="n">
-        <v>190198</v>
+        <v>211981</v>
       </c>
       <c r="E16" s="12" t="n">
-        <v>0.67</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="F16" t="n">
-        <v>1.24</v>
+        <v>1.29</v>
       </c>
       <c r="G16" t="n">
-        <v>3307</v>
+        <v>4109</v>
       </c>
       <c r="H16" s="12" t="n">
         <v>0.04</v>
       </c>
       <c r="I16" s="13" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="J16" t="n">
+        <v>45</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <v>3.23</v>
+      </c>
+      <c r="L16" s="12" t="n">
+        <v>58.12</v>
+      </c>
+      <c r="Q16" s="12" t="n"/>
+      <c r="S16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-13</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>127.52</v>
+      </c>
+      <c r="C17" t="n">
+        <v>154355</v>
+      </c>
+      <c r="D17" t="n">
+        <v>190813</v>
+      </c>
+      <c r="E17" s="12" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="G17" t="n">
+        <v>3321</v>
+      </c>
+      <c r="H17" s="12" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="I17" s="13" t="n">
         <v>1.74</v>
       </c>
-      <c r="N16" s="12" t="n"/>
-      <c r="P16" s="13" t="n"/>
+      <c r="J17" t="n">
+        <v>29</v>
+      </c>
+      <c r="K17" s="12" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="L17" s="12" t="n">
+        <v>35.41</v>
+      </c>
+      <c r="Q17" s="12" t="n"/>
+      <c r="S17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>72.08</v>
+      </c>
+      <c r="C18" t="n">
+        <v>114773</v>
+      </c>
+      <c r="D18" t="n">
+        <v>126674</v>
+      </c>
+      <c r="E18" s="12" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="G18" t="n">
+        <v>1572</v>
+      </c>
+      <c r="H18" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I18" s="13" t="n">
+        <v>1.24</v>
+      </c>
+      <c r="J18" t="n">
+        <v>13</v>
+      </c>
+      <c r="K18" s="12" t="n">
+        <v>5.54</v>
+      </c>
+      <c r="L18" s="12" t="n"/>
+      <c r="Q18" s="12" t="n"/>
+      <c r="S18" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>88.95999999999999</v>
+      </c>
+      <c r="C19" t="n">
+        <v>112804</v>
+      </c>
+      <c r="D19" t="n">
+        <v>130486</v>
+      </c>
+      <c r="E19" s="12" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1973</v>
+      </c>
+      <c r="H19" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I19" s="13" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="J19" t="n">
+        <v>7</v>
+      </c>
+      <c r="K19" s="12" t="n">
+        <v>12.71</v>
+      </c>
+      <c r="L19" s="12" t="n">
+        <v>128.76</v>
+      </c>
+      <c r="Q19" s="12" t="n"/>
+      <c r="S19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="n">
+        <v>120.01</v>
+      </c>
+      <c r="C20" t="n">
+        <v>203373</v>
+      </c>
+      <c r="D20" t="n">
+        <v>225405</v>
+      </c>
+      <c r="E20" s="12" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="G20" t="n">
+        <v>2372</v>
+      </c>
+      <c r="H20" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I20" s="13" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="J20" t="n">
+        <v>12</v>
+      </c>
+      <c r="K20" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="L20" s="12" t="n">
+        <v>39.07</v>
+      </c>
+      <c r="Q20" s="12" t="n"/>
+      <c r="S20" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A1:S1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -3166,7 +3954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N17"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3283,47 +4071,47 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>2026-04-01 → 2026-04-13</t>
+          <t>2026-04-01 → 2026-04-16</t>
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>2512.980000000001</v>
+        <v>2994.370000000001</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>528398</v>
+        <v>681032</v>
       </c>
       <c r="D4" s="8" t="n">
-        <v>4.76</v>
+        <v>4.4</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>34906</v>
+        <v>43634</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>6.61</v>
+        <v>6.41</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>31563</v>
+        <v>39761</v>
       </c>
       <c r="I4" s="7" t="n">
-        <v>2591</v>
+        <v>3198</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>1124</v>
+        <v>1361</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>152</v>
+        <v>185</v>
       </c>
       <c r="L4" s="8" t="n">
-        <v>7526.614465000001</v>
+        <v>9187.598484999999</v>
       </c>
       <c r="M4" s="7" t="n">
-        <v>3</v>
+        <v>3.07</v>
       </c>
       <c r="N4" s="9" t="n">
-        <v>0.48</v>
+        <v>0.47</v>
       </c>
     </row>
     <row r="5">
@@ -3676,6 +4464,87 @@
       </c>
       <c r="L17" s="12" t="n"/>
       <c r="N17" s="13" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-04-14</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>171.26</v>
+      </c>
+      <c r="C18" t="n">
+        <v>53464</v>
+      </c>
+      <c r="D18" s="12" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3014</v>
+      </c>
+      <c r="F18" s="12" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G18" s="13" t="n">
+        <v>5.64</v>
+      </c>
+      <c r="L18" s="12" t="n"/>
+      <c r="N18" s="13" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-04-15</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>175.6499999999999</v>
+      </c>
+      <c r="C19" t="n">
+        <v>51569</v>
+      </c>
+      <c r="D19" s="12" t="n">
+        <v>3.41</v>
+      </c>
+      <c r="E19" t="n">
+        <v>2963</v>
+      </c>
+      <c r="F19" s="12" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G19" s="13" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="L19" s="12" t="n"/>
+      <c r="N19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="n">
+        <v>134.48</v>
+      </c>
+      <c r="C20" t="n">
+        <v>47604</v>
+      </c>
+      <c r="D20" s="12" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2751</v>
+      </c>
+      <c r="F20" s="12" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="L20" s="12" t="n"/>
+      <c r="N20" s="13" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6196,4 +7065,1193 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AD26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="14" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
+    <col width="14" customWidth="1" min="30" max="30"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="48" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MOSCA HNOS.  ·  Reporte 01/04/2026 → 17/04/2026  </t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="6" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Campaña</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Inversión</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Alcance</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Impr.</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>CPM</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Frec.</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>CPC</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>CTR</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Usuarios GA4</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Sesiones</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>Add Cart</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>Checkout</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>Compras</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>ROAS</t>
+        </is>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>Conv.%</t>
+        </is>
+      </c>
+      <c r="R3" s="3" t="inlineStr">
+        <is>
+          <t>Compras Meta</t>
+        </is>
+      </c>
+      <c r="S3" s="3" t="inlineStr">
+        <is>
+          <t>CPA Meta</t>
+        </is>
+      </c>
+      <c r="T3" s="3" t="inlineStr">
+        <is>
+          <t>Valor Meta</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL PERÍODO</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="n">
+        <v>4950.22</v>
+      </c>
+      <c r="C4" s="16" t="n">
+        <v>828107</v>
+      </c>
+      <c r="D4" s="16" t="n">
+        <v>3668887</v>
+      </c>
+      <c r="E4" s="15" t="n">
+        <v>1.349242972051197</v>
+      </c>
+      <c r="F4" s="16" t="n"/>
+      <c r="G4" s="16" t="n">
+        <v>99151</v>
+      </c>
+      <c r="H4" s="15" t="n">
+        <v>0.04992607235428791</v>
+      </c>
+      <c r="I4" s="17" t="n"/>
+      <c r="J4" s="16" t="n"/>
+      <c r="K4" s="16" t="n"/>
+      <c r="L4" s="16" t="n"/>
+      <c r="M4" s="16" t="n"/>
+      <c r="N4" s="16" t="n"/>
+      <c r="O4" s="15" t="n"/>
+      <c r="P4" s="16" t="n"/>
+      <c r="Q4" s="17" t="n"/>
+      <c r="R4" s="16" t="n">
+        <v>333</v>
+      </c>
+      <c r="S4" s="15" t="n">
+        <v>14.87</v>
+      </c>
+      <c r="T4" s="15" t="n">
+        <v>529.03</v>
+      </c>
+      <c r="Z4" s="18" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="AA4" s="18" t="inlineStr">
+        <is>
+          <t>Inversión</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="19" t="inlineStr">
+        <is>
+          <t>META ADS  ·  7 campañas</t>
+        </is>
+      </c>
+      <c r="B5" s="20" t="n">
+        <v>1939.81</v>
+      </c>
+      <c r="C5" s="21" t="n">
+        <v>828107</v>
+      </c>
+      <c r="D5" s="21" t="n">
+        <v>2980100</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>0.6509211100298649</v>
+      </c>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="21" t="n">
+        <v>55131</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>0.03518546734142316</v>
+      </c>
+      <c r="I5" s="22" t="n"/>
+      <c r="J5" s="21" t="n"/>
+      <c r="K5" s="21" t="n"/>
+      <c r="L5" s="21" t="n"/>
+      <c r="M5" s="21" t="n"/>
+      <c r="N5" s="21" t="n"/>
+      <c r="O5" s="20" t="n"/>
+      <c r="P5" s="21" t="n"/>
+      <c r="Q5" s="22" t="n"/>
+      <c r="R5" s="21" t="n">
+        <v>333</v>
+      </c>
+      <c r="S5" s="20" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="T5" s="20" t="n">
+        <v>529.03</v>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="AA5" s="12" t="n">
+        <v>1939.81</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>Meta | Alcance</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="n">
+        <v>213.02</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <v>265446</v>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>783389</v>
+      </c>
+      <c r="E6" s="24" t="n">
+        <v>0.271921</v>
+      </c>
+      <c r="F6" s="25" t="n">
+        <v>2.951218</v>
+      </c>
+      <c r="G6" s="25" t="n">
+        <v>2106</v>
+      </c>
+      <c r="H6" s="24" t="n">
+        <v>0.101149</v>
+      </c>
+      <c r="I6" s="26" t="n">
+        <v>0.268832</v>
+      </c>
+      <c r="J6" s="25" t="n"/>
+      <c r="K6" s="25" t="n"/>
+      <c r="L6" s="25" t="n"/>
+      <c r="M6" s="25" t="n"/>
+      <c r="N6" s="25" t="n"/>
+      <c r="O6" s="24" t="n"/>
+      <c r="P6" s="25" t="n"/>
+      <c r="Q6" s="26" t="n"/>
+      <c r="R6" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="S6" s="24" t="n">
+        <v>16.39</v>
+      </c>
+      <c r="T6" s="24" t="n">
+        <v>56.29</v>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="AA6" s="12" t="n">
+        <v>3010.41</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="inlineStr">
+        <is>
+          <t>Meta | Alcance | Interior</t>
+        </is>
+      </c>
+      <c r="B7" s="28" t="n">
+        <v>195.67</v>
+      </c>
+      <c r="C7" s="29" t="n">
+        <v>273166</v>
+      </c>
+      <c r="D7" s="29" t="n">
+        <v>857870</v>
+      </c>
+      <c r="E7" s="28" t="n">
+        <v>0.228088</v>
+      </c>
+      <c r="F7" s="29" t="n">
+        <v>3.140471</v>
+      </c>
+      <c r="G7" s="29" t="n">
+        <v>1852</v>
+      </c>
+      <c r="H7" s="28" t="n">
+        <v>0.105653</v>
+      </c>
+      <c r="I7" s="30" t="n">
+        <v>0.215884</v>
+      </c>
+      <c r="J7" s="29" t="n"/>
+      <c r="K7" s="29" t="n"/>
+      <c r="L7" s="29" t="n"/>
+      <c r="M7" s="29" t="n"/>
+      <c r="N7" s="29" t="n"/>
+      <c r="O7" s="28" t="n"/>
+      <c r="P7" s="29" t="n"/>
+      <c r="Q7" s="30" t="n"/>
+      <c r="R7" s="29" t="n"/>
+      <c r="S7" s="28" t="n"/>
+      <c r="T7" s="28" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>Meta | Clientes potenciales | HOY Beneficios</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="n">
+        <v>42.44</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>7767</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>12498</v>
+      </c>
+      <c r="E8" s="24" t="n">
+        <v>3.395743</v>
+      </c>
+      <c r="F8" s="25" t="n">
+        <v>1.609115</v>
+      </c>
+      <c r="G8" s="25" t="n">
+        <v>248</v>
+      </c>
+      <c r="H8" s="24" t="n">
+        <v>0.171129</v>
+      </c>
+      <c r="I8" s="26" t="n">
+        <v>1.984317</v>
+      </c>
+      <c r="J8" s="25" t="n"/>
+      <c r="K8" s="25" t="n"/>
+      <c r="L8" s="25" t="n"/>
+      <c r="M8" s="25" t="n"/>
+      <c r="N8" s="25" t="n"/>
+      <c r="O8" s="24" t="n"/>
+      <c r="P8" s="25" t="n"/>
+      <c r="Q8" s="26" t="n"/>
+      <c r="R8" s="25" t="n"/>
+      <c r="S8" s="24" t="n"/>
+      <c r="T8" s="24" t="n"/>
+      <c r="Z8" s="18" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="AA8" s="18" t="inlineStr">
+        <is>
+          <t>Impresiones</t>
+        </is>
+      </c>
+      <c r="AC8" s="18" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="AD8" s="18" t="inlineStr">
+        <is>
+          <t>CPM</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="27" t="inlineStr">
+        <is>
+          <t>Meta | Ventas | AO | Remarketing</t>
+        </is>
+      </c>
+      <c r="B9" s="28" t="n">
+        <v>235.31</v>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>23136</v>
+      </c>
+      <c r="D9" s="29" t="n">
+        <v>104003</v>
+      </c>
+      <c r="E9" s="28" t="n">
+        <v>2.262531</v>
+      </c>
+      <c r="F9" s="29" t="n">
+        <v>4.495289</v>
+      </c>
+      <c r="G9" s="29" t="n">
+        <v>4217</v>
+      </c>
+      <c r="H9" s="28" t="n">
+        <v>0.0558</v>
+      </c>
+      <c r="I9" s="30" t="n">
+        <v>4.054691</v>
+      </c>
+      <c r="J9" s="29" t="n"/>
+      <c r="K9" s="29" t="n"/>
+      <c r="L9" s="29" t="n"/>
+      <c r="M9" s="29" t="n"/>
+      <c r="N9" s="29" t="n"/>
+      <c r="O9" s="28" t="n"/>
+      <c r="P9" s="29" t="n"/>
+      <c r="Q9" s="30" t="n"/>
+      <c r="R9" s="29" t="n">
+        <v>228</v>
+      </c>
+      <c r="S9" s="28" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="T9" s="28" t="n">
+        <v>350.6</v>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="AA9" t="n">
+        <v>2980100</v>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="AD9" s="12" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="23" t="inlineStr">
+        <is>
+          <t>Meta | Conversión | (CONV)</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="C10" s="25" t="n">
+        <v>17451</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>35393</v>
+      </c>
+      <c r="E10" s="24" t="n">
+        <v>1.738479</v>
+      </c>
+      <c r="F10" s="25" t="n">
+        <v>2.028136</v>
+      </c>
+      <c r="G10" s="25" t="n">
+        <v>1050</v>
+      </c>
+      <c r="H10" s="24" t="n">
+        <v>0.0586</v>
+      </c>
+      <c r="I10" s="26" t="n">
+        <v>2.966688</v>
+      </c>
+      <c r="J10" s="25" t="n"/>
+      <c r="K10" s="25" t="n"/>
+      <c r="L10" s="25" t="n"/>
+      <c r="M10" s="25" t="n"/>
+      <c r="N10" s="25" t="n"/>
+      <c r="O10" s="24" t="n"/>
+      <c r="P10" s="25" t="n"/>
+      <c r="Q10" s="26" t="n"/>
+      <c r="R10" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="S10" s="24" t="n">
+        <v>30.77</v>
+      </c>
+      <c r="T10" s="24" t="n">
+        <v>72.47</v>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="AA10" t="n">
+        <v>688787</v>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="AD10" s="12" t="n">
+        <v>4.37</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Meta | Tráfico</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="n">
+        <v>1141.96</v>
+      </c>
+      <c r="C11" s="29" t="n">
+        <v>211812</v>
+      </c>
+      <c r="D11" s="29" t="n">
+        <v>1117030</v>
+      </c>
+      <c r="E11" s="28" t="n">
+        <v>1.022318</v>
+      </c>
+      <c r="F11" s="29" t="n">
+        <v>5.273686</v>
+      </c>
+      <c r="G11" s="29" t="n">
+        <v>38724</v>
+      </c>
+      <c r="H11" s="28" t="n">
+        <v>0.02949</v>
+      </c>
+      <c r="I11" s="30" t="n">
+        <v>3.466693</v>
+      </c>
+      <c r="J11" s="29" t="n"/>
+      <c r="K11" s="29" t="n"/>
+      <c r="L11" s="29" t="n"/>
+      <c r="M11" s="29" t="n"/>
+      <c r="N11" s="29" t="n"/>
+      <c r="O11" s="28" t="n"/>
+      <c r="P11" s="29" t="n"/>
+      <c r="Q11" s="30" t="n"/>
+      <c r="R11" s="29" t="n">
+        <v>90</v>
+      </c>
+      <c r="S11" s="28" t="n">
+        <v>12.69</v>
+      </c>
+      <c r="T11" s="28" t="n">
+        <v>49.67</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Tráfico Campaña RRHH</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="n">
+        <v>49.88</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>29329</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>69917</v>
+      </c>
+      <c r="E12" s="24" t="n">
+        <v>0.713417</v>
+      </c>
+      <c r="F12" s="25" t="n">
+        <v>2.383886</v>
+      </c>
+      <c r="G12" s="25" t="n">
+        <v>6934</v>
+      </c>
+      <c r="H12" s="24" t="n">
+        <v>0.007194</v>
+      </c>
+      <c r="I12" s="26" t="n">
+        <v>9.917474</v>
+      </c>
+      <c r="J12" s="25" t="n"/>
+      <c r="K12" s="25" t="n"/>
+      <c r="L12" s="25" t="n"/>
+      <c r="M12" s="25" t="n"/>
+      <c r="N12" s="25" t="n"/>
+      <c r="O12" s="24" t="n"/>
+      <c r="P12" s="25" t="n"/>
+      <c r="Q12" s="26" t="n"/>
+      <c r="R12" s="25" t="n"/>
+      <c r="S12" s="24" t="n"/>
+      <c r="T12" s="24" t="n"/>
+      <c r="Z12" s="18" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="AA12" s="18" t="inlineStr">
+        <is>
+          <t>Clicks</t>
+        </is>
+      </c>
+      <c r="AC12" s="18" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="AD12" s="18" t="inlineStr">
+        <is>
+          <t>CPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>GOOGLE ADS  ·  8 campañas</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="n">
+        <v>3010.41</v>
+      </c>
+      <c r="C13" s="33" t="n"/>
+      <c r="D13" s="33" t="n">
+        <v>688787</v>
+      </c>
+      <c r="E13" s="32" t="n">
+        <v>4.370596425310001</v>
+      </c>
+      <c r="F13" s="33" t="n"/>
+      <c r="G13" s="33" t="n">
+        <v>44020</v>
+      </c>
+      <c r="H13" s="32" t="n">
+        <v>0.06838732394366197</v>
+      </c>
+      <c r="I13" s="34" t="n"/>
+      <c r="J13" s="33" t="n"/>
+      <c r="K13" s="33" t="n"/>
+      <c r="L13" s="33" t="n"/>
+      <c r="M13" s="33" t="n"/>
+      <c r="N13" s="33" t="n"/>
+      <c r="O13" s="32" t="n"/>
+      <c r="P13" s="33" t="n"/>
+      <c r="Q13" s="34" t="n"/>
+      <c r="R13" s="33" t="n"/>
+      <c r="S13" s="32" t="n"/>
+      <c r="T13" s="32" t="n"/>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="AA13" t="n">
+        <v>55131</v>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="AD13" s="12" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="23" t="inlineStr">
+        <is>
+          <t>PMax (CONV)</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="n">
+        <v>453.98</v>
+      </c>
+      <c r="C14" s="25" t="n"/>
+      <c r="D14" s="25" t="n">
+        <v>154176</v>
+      </c>
+      <c r="E14" s="24" t="n">
+        <v>2.94</v>
+      </c>
+      <c r="F14" s="25" t="n"/>
+      <c r="G14" s="25" t="n">
+        <v>7376</v>
+      </c>
+      <c r="H14" s="24" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I14" s="26" t="n">
+        <v>4.78</v>
+      </c>
+      <c r="J14" s="25" t="n"/>
+      <c r="K14" s="25" t="n"/>
+      <c r="L14" s="25" t="n"/>
+      <c r="M14" s="25" t="n"/>
+      <c r="N14" s="25" t="n"/>
+      <c r="O14" s="24" t="n"/>
+      <c r="P14" s="25" t="n"/>
+      <c r="Q14" s="26" t="n"/>
+      <c r="R14" s="25" t="n"/>
+      <c r="S14" s="24" t="n"/>
+      <c r="T14" s="24" t="n"/>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="AA14" t="n">
+        <v>44020</v>
+      </c>
+      <c r="AC14" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="AD14" s="12" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>Search | Brand (CONV)</t>
+        </is>
+      </c>
+      <c r="B15" s="28" t="n">
+        <v>1258.98</v>
+      </c>
+      <c r="C15" s="29" t="n"/>
+      <c r="D15" s="29" t="n">
+        <v>57840</v>
+      </c>
+      <c r="E15" s="28" t="n">
+        <v>21.77</v>
+      </c>
+      <c r="F15" s="29" t="n"/>
+      <c r="G15" s="29" t="n">
+        <v>19430</v>
+      </c>
+      <c r="H15" s="28" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I15" s="30" t="n">
+        <v>33.59</v>
+      </c>
+      <c r="J15" s="29" t="n"/>
+      <c r="K15" s="29" t="n"/>
+      <c r="L15" s="29" t="n"/>
+      <c r="M15" s="29" t="n"/>
+      <c r="N15" s="29" t="n"/>
+      <c r="O15" s="28" t="n"/>
+      <c r="P15" s="29" t="n"/>
+      <c r="Q15" s="30" t="n"/>
+      <c r="R15" s="29" t="n"/>
+      <c r="S15" s="28" t="n"/>
+      <c r="T15" s="28" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>Search | Genérico | Juguetes</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="n">
+        <v>242.62</v>
+      </c>
+      <c r="C16" s="25" t="n"/>
+      <c r="D16" s="25" t="n">
+        <v>53513</v>
+      </c>
+      <c r="E16" s="24" t="n">
+        <v>4.53</v>
+      </c>
+      <c r="F16" s="25" t="n"/>
+      <c r="G16" s="25" t="n">
+        <v>1926</v>
+      </c>
+      <c r="H16" s="24" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="I16" s="26" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J16" s="25" t="n"/>
+      <c r="K16" s="25" t="n"/>
+      <c r="L16" s="25" t="n"/>
+      <c r="M16" s="25" t="n"/>
+      <c r="N16" s="25" t="n"/>
+      <c r="O16" s="24" t="n"/>
+      <c r="P16" s="25" t="n"/>
+      <c r="Q16" s="26" t="n"/>
+      <c r="R16" s="25" t="n"/>
+      <c r="S16" s="24" t="n"/>
+      <c r="T16" s="24" t="n"/>
+      <c r="Z16" s="18" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="AA16" s="18" t="inlineStr">
+        <is>
+          <t>Sesiones</t>
+        </is>
+      </c>
+      <c r="AC16" s="18" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="AD16" s="18" t="inlineStr">
+        <is>
+          <t>Costo/Sesión</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>Search | Genérica | Arte</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="n">
+        <v>227.4</v>
+      </c>
+      <c r="C17" s="29" t="n"/>
+      <c r="D17" s="29" t="n">
+        <v>16690</v>
+      </c>
+      <c r="E17" s="28" t="n">
+        <v>13.63</v>
+      </c>
+      <c r="F17" s="29" t="n"/>
+      <c r="G17" s="29" t="n">
+        <v>1115</v>
+      </c>
+      <c r="H17" s="28" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="I17" s="30" t="n">
+        <v>6.68</v>
+      </c>
+      <c r="J17" s="29" t="n"/>
+      <c r="K17" s="29" t="n"/>
+      <c r="L17" s="29" t="n"/>
+      <c r="M17" s="29" t="n"/>
+      <c r="N17" s="29" t="n"/>
+      <c r="O17" s="28" t="n"/>
+      <c r="P17" s="29" t="n"/>
+      <c r="Q17" s="30" t="n"/>
+      <c r="R17" s="29" t="n"/>
+      <c r="S17" s="28" t="n"/>
+      <c r="T17" s="28" t="n"/>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="AA17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC17" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="AD17" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="inlineStr">
+        <is>
+          <t>Search | Primera infancia</t>
+        </is>
+      </c>
+      <c r="B18" s="24" t="n">
+        <v>114.85</v>
+      </c>
+      <c r="C18" s="25" t="n"/>
+      <c r="D18" s="25" t="n">
+        <v>13492</v>
+      </c>
+      <c r="E18" s="24" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n">
+        <v>871</v>
+      </c>
+      <c r="H18" s="24" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="I18" s="26" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="J18" s="25" t="n"/>
+      <c r="K18" s="25" t="n"/>
+      <c r="L18" s="25" t="n"/>
+      <c r="M18" s="25" t="n"/>
+      <c r="N18" s="25" t="n"/>
+      <c r="O18" s="24" t="n"/>
+      <c r="P18" s="25" t="n"/>
+      <c r="Q18" s="26" t="n"/>
+      <c r="R18" s="25" t="n"/>
+      <c r="S18" s="24" t="n"/>
+      <c r="T18" s="24" t="n"/>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="AA18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="AD18" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>Search | Brand | La papelaria</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="n">
+        <v>56.16</v>
+      </c>
+      <c r="C19" s="29" t="n"/>
+      <c r="D19" s="29" t="n">
+        <v>7520</v>
+      </c>
+      <c r="E19" s="28" t="n">
+        <v>7.47</v>
+      </c>
+      <c r="F19" s="29" t="n"/>
+      <c r="G19" s="29" t="n">
+        <v>652</v>
+      </c>
+      <c r="H19" s="28" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="I19" s="30" t="n">
+        <v>8.67</v>
+      </c>
+      <c r="J19" s="29" t="n"/>
+      <c r="K19" s="29" t="n"/>
+      <c r="L19" s="29" t="n"/>
+      <c r="M19" s="29" t="n"/>
+      <c r="N19" s="29" t="n"/>
+      <c r="O19" s="28" t="n"/>
+      <c r="P19" s="29" t="n"/>
+      <c r="Q19" s="30" t="n"/>
+      <c r="R19" s="29" t="n"/>
+      <c r="S19" s="28" t="n"/>
+      <c r="T19" s="28" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>Search | Genérico | Tecnología</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="n">
+        <v>53.91</v>
+      </c>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n">
+        <v>15255</v>
+      </c>
+      <c r="E20" s="24" t="n">
+        <v>3.53</v>
+      </c>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n">
+        <v>561</v>
+      </c>
+      <c r="H20" s="24" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I20" s="26" t="n">
+        <v>3.68</v>
+      </c>
+      <c r="J20" s="25" t="n"/>
+      <c r="K20" s="25" t="n"/>
+      <c r="L20" s="25" t="n"/>
+      <c r="M20" s="25" t="n"/>
+      <c r="N20" s="25" t="n"/>
+      <c r="O20" s="24" t="n"/>
+      <c r="P20" s="25" t="n"/>
+      <c r="Q20" s="26" t="n"/>
+      <c r="R20" s="25" t="n"/>
+      <c r="S20" s="24" t="n"/>
+      <c r="T20" s="24" t="n"/>
+      <c r="Z20" s="18" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="AA20" s="18" t="inlineStr">
+        <is>
+          <t>Compras</t>
+        </is>
+      </c>
+      <c r="AC20" s="18" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="AD20" s="18" t="inlineStr">
+        <is>
+          <t>CPA</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>Shopping (CONV)</t>
+        </is>
+      </c>
+      <c r="B21" s="28" t="n">
+        <v>602.51</v>
+      </c>
+      <c r="C21" s="29" t="n"/>
+      <c r="D21" s="29" t="n">
+        <v>370301</v>
+      </c>
+      <c r="E21" s="28" t="n">
+        <v>1.63</v>
+      </c>
+      <c r="F21" s="29" t="n"/>
+      <c r="G21" s="29" t="n">
+        <v>12089</v>
+      </c>
+      <c r="H21" s="28" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I21" s="30" t="n">
+        <v>3.26</v>
+      </c>
+      <c r="J21" s="29" t="n"/>
+      <c r="K21" s="29" t="n"/>
+      <c r="L21" s="29" t="n"/>
+      <c r="M21" s="29" t="n"/>
+      <c r="N21" s="29" t="n"/>
+      <c r="O21" s="28" t="n"/>
+      <c r="P21" s="29" t="n"/>
+      <c r="Q21" s="30" t="n"/>
+      <c r="R21" s="29" t="n"/>
+      <c r="S21" s="28" t="n"/>
+      <c r="T21" s="28" t="n"/>
+      <c r="Z21" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="AA21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="AD21" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="AA22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="AD22" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="Z24" s="18" t="inlineStr">
+        <is>
+          <t>Plataforma</t>
+        </is>
+      </c>
+      <c r="AA24" s="18" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>Meta Ads</t>
+        </is>
+      </c>
+      <c r="AA25" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>Google Ads</t>
+        </is>
+      </c>
+      <c r="AA26" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:T1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Documenta operación y corrige actualización de status GA4
- Agrega README.md con configuración y mantenimiento operativo.
- Regenera siempre la pestaña diaria de status para actualizar GA4.
- Actualiza el Excel mensual con la pestaña 17-04-2026 corregida.

Co-Authored-By: Oz <oz-agent@warp.dev>
</commit_message>
<xml_diff>
--- a/reporter/Mosca | Performance | Reporte mensual 2026-04.xlsx
+++ b/reporter/Mosca | Performance | Reporte mensual 2026-04.xlsx
@@ -625,6 +625,7 @@
 
 <file path=xl/charts/chart13.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -689,6 +690,7 @@
 
 <file path=xl/charts/chart14.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -753,6 +755,7 @@
 
 <file path=xl/charts/chart15.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -817,6 +820,7 @@
 
 <file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -881,6 +885,7 @@
 
 <file path=xl/charts/chart17.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -945,6 +950,7 @@
 
 <file path=xl/charts/chart18.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="2"/>
   <chart>
     <title>
       <tx>
@@ -2103,9 +2109,6 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
-        <a:ln>
-          <a:prstDash val="solid"/>
-        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -2537,7 +2540,7 @@
         <v>354</v>
       </c>
       <c r="F5" s="15" t="n">
-        <v>4901.079999999999</v>
+        <v>4901.15</v>
       </c>
       <c r="G5" s="15" t="n">
         <v>18597.882743</v>
@@ -3245,13 +3248,13 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>1906.71</v>
+        <v>1906.78</v>
       </c>
       <c r="C4" s="7" t="n">
-        <v>2307936</v>
+        <v>2307966</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>2919715</v>
+        <v>2919779</v>
       </c>
       <c r="E4" s="8" t="n">
         <v>0.65</v>
@@ -4084,7 +4087,7 @@
         <v>4.4</v>
       </c>
       <c r="E4" s="7" t="n">
-        <v>43634</v>
+        <v>43633</v>
       </c>
       <c r="F4" s="8" t="n">
         <v>0.07000000000000001</v>
@@ -7240,38 +7243,54 @@
         </is>
       </c>
       <c r="B4" s="15" t="n">
-        <v>4950.22</v>
+        <v>4980.25</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>828107</v>
+        <v>832660</v>
       </c>
       <c r="D4" s="16" t="n">
-        <v>3668887</v>
+        <v>3691398</v>
       </c>
       <c r="E4" s="15" t="n">
-        <v>1.349242972051197</v>
+        <v>1.3491501051905</v>
       </c>
       <c r="F4" s="16" t="n"/>
       <c r="G4" s="16" t="n">
-        <v>99151</v>
+        <v>99664</v>
       </c>
       <c r="H4" s="15" t="n">
-        <v>0.04992607235428791</v>
+        <v>0.049970400545834</v>
       </c>
       <c r="I4" s="17" t="n"/>
-      <c r="J4" s="16" t="n"/>
-      <c r="K4" s="16" t="n"/>
-      <c r="L4" s="16" t="n"/>
-      <c r="M4" s="16" t="n"/>
-      <c r="N4" s="16" t="n"/>
-      <c r="O4" s="15" t="n"/>
-      <c r="P4" s="16" t="n"/>
-      <c r="Q4" s="17" t="n"/>
+      <c r="J4" s="16" t="n">
+        <v>41620</v>
+      </c>
+      <c r="K4" s="16" t="n">
+        <v>52734</v>
+      </c>
+      <c r="L4" s="16" t="n">
+        <v>3576</v>
+      </c>
+      <c r="M4" s="16" t="n">
+        <v>1460</v>
+      </c>
+      <c r="N4" s="16" t="n">
+        <v>195</v>
+      </c>
+      <c r="O4" s="15" t="n">
+        <v>9575.076480999998</v>
+      </c>
+      <c r="P4" s="16" t="n">
+        <v>1.922609604136338</v>
+      </c>
+      <c r="Q4" s="17" t="n">
+        <v>0.369780407327341</v>
+      </c>
       <c r="R4" s="16" t="n">
         <v>333</v>
       </c>
       <c r="S4" s="15" t="n">
-        <v>14.87</v>
+        <v>14.96</v>
       </c>
       <c r="T4" s="15" t="n">
         <v>529.03</v>
@@ -7294,38 +7313,54 @@
         </is>
       </c>
       <c r="B5" s="20" t="n">
-        <v>1939.81</v>
+        <v>1951.12</v>
       </c>
       <c r="C5" s="21" t="n">
-        <v>828107</v>
+        <v>832660</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>2980100</v>
+        <v>2997795</v>
       </c>
       <c r="E5" s="20" t="n">
-        <v>0.6509211100298649</v>
+        <v>0.6508517093396982</v>
       </c>
       <c r="F5" s="21" t="n"/>
       <c r="G5" s="21" t="n">
-        <v>55131</v>
+        <v>55313</v>
       </c>
       <c r="H5" s="20" t="n">
-        <v>0.03518546734142316</v>
+        <v>0.03527416701317955</v>
       </c>
       <c r="I5" s="22" t="n"/>
-      <c r="J5" s="21" t="n"/>
-      <c r="K5" s="21" t="n"/>
-      <c r="L5" s="21" t="n"/>
-      <c r="M5" s="21" t="n"/>
-      <c r="N5" s="21" t="n"/>
-      <c r="O5" s="20" t="n"/>
-      <c r="P5" s="21" t="n"/>
-      <c r="Q5" s="22" t="n"/>
+      <c r="J5" s="21" t="n">
+        <v>10523</v>
+      </c>
+      <c r="K5" s="21" t="n">
+        <v>12684</v>
+      </c>
+      <c r="L5" s="21" t="n">
+        <v>339</v>
+      </c>
+      <c r="M5" s="21" t="n">
+        <v>97</v>
+      </c>
+      <c r="N5" s="21" t="n">
+        <v>10</v>
+      </c>
+      <c r="O5" s="20" t="n">
+        <v>387.477996</v>
+      </c>
+      <c r="P5" s="21" t="n">
+        <v>0.1985926011726598</v>
+      </c>
+      <c r="Q5" s="22" t="n">
+        <v>0.07883948281299274</v>
+      </c>
       <c r="R5" s="21" t="n">
         <v>333</v>
       </c>
       <c r="S5" s="20" t="n">
-        <v>5.83</v>
+        <v>5.86</v>
       </c>
       <c r="T5" s="20" t="n">
         <v>529.03</v>
@@ -7336,7 +7371,7 @@
         </is>
       </c>
       <c r="AA5" s="12" t="n">
-        <v>1939.81</v>
+        <v>1951.12</v>
       </c>
     </row>
     <row r="6">
@@ -7346,42 +7381,48 @@
         </is>
       </c>
       <c r="B6" s="24" t="n">
-        <v>213.02</v>
+        <v>216</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>265446</v>
+        <v>269090</v>
       </c>
       <c r="D6" s="25" t="n">
-        <v>783389</v>
+        <v>791746</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>0.271921</v>
+        <v>0.272815</v>
       </c>
       <c r="F6" s="25" t="n">
-        <v>2.951218</v>
+        <v>2.942309</v>
       </c>
       <c r="G6" s="25" t="n">
-        <v>2106</v>
+        <v>2130</v>
       </c>
       <c r="H6" s="24" t="n">
-        <v>0.101149</v>
+        <v>0.101408</v>
       </c>
       <c r="I6" s="26" t="n">
-        <v>0.268832</v>
-      </c>
-      <c r="J6" s="25" t="n"/>
-      <c r="K6" s="25" t="n"/>
+        <v>0.269026</v>
+      </c>
+      <c r="J6" s="25" t="n">
+        <v>183</v>
+      </c>
+      <c r="K6" s="25" t="n">
+        <v>193</v>
+      </c>
       <c r="L6" s="25" t="n"/>
       <c r="M6" s="25" t="n"/>
       <c r="N6" s="25" t="n"/>
       <c r="O6" s="24" t="n"/>
       <c r="P6" s="25" t="n"/>
-      <c r="Q6" s="26" t="n"/>
+      <c r="Q6" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="R6" s="25" t="n">
         <v>13</v>
       </c>
       <c r="S6" s="24" t="n">
-        <v>16.39</v>
+        <v>16.62</v>
       </c>
       <c r="T6" s="24" t="n">
         <v>56.29</v>
@@ -7392,7 +7433,7 @@
         </is>
       </c>
       <c r="AA6" s="12" t="n">
-        <v>3010.41</v>
+        <v>3029.13</v>
       </c>
     </row>
     <row r="7">
@@ -7402,37 +7443,43 @@
         </is>
       </c>
       <c r="B7" s="28" t="n">
-        <v>195.67</v>
+        <v>196.85</v>
       </c>
       <c r="C7" s="29" t="n">
-        <v>273166</v>
+        <v>273359</v>
       </c>
       <c r="D7" s="29" t="n">
-        <v>857870</v>
+        <v>862668</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>0.228088</v>
+        <v>0.228187</v>
       </c>
       <c r="F7" s="29" t="n">
-        <v>3.140471</v>
+        <v>3.155806</v>
       </c>
       <c r="G7" s="29" t="n">
-        <v>1852</v>
+        <v>1863</v>
       </c>
       <c r="H7" s="28" t="n">
-        <v>0.105653</v>
+        <v>0.105663</v>
       </c>
       <c r="I7" s="30" t="n">
-        <v>0.215884</v>
-      </c>
-      <c r="J7" s="29" t="n"/>
-      <c r="K7" s="29" t="n"/>
+        <v>0.215958</v>
+      </c>
+      <c r="J7" s="29" t="n">
+        <v>183</v>
+      </c>
+      <c r="K7" s="29" t="n">
+        <v>193</v>
+      </c>
       <c r="L7" s="29" t="n"/>
       <c r="M7" s="29" t="n"/>
       <c r="N7" s="29" t="n"/>
       <c r="O7" s="28" t="n"/>
       <c r="P7" s="29" t="n"/>
-      <c r="Q7" s="30" t="n"/>
+      <c r="Q7" s="30" t="n">
+        <v>0</v>
+      </c>
       <c r="R7" s="29" t="n"/>
       <c r="S7" s="28" t="n"/>
       <c r="T7" s="28" t="n"/>
@@ -7467,14 +7514,20 @@
       <c r="I8" s="26" t="n">
         <v>1.984317</v>
       </c>
-      <c r="J8" s="25" t="n"/>
-      <c r="K8" s="25" t="n"/>
+      <c r="J8" s="25" t="n">
+        <v>128</v>
+      </c>
+      <c r="K8" s="25" t="n">
+        <v>136</v>
+      </c>
       <c r="L8" s="25" t="n"/>
       <c r="M8" s="25" t="n"/>
       <c r="N8" s="25" t="n"/>
       <c r="O8" s="24" t="n"/>
       <c r="P8" s="25" t="n"/>
-      <c r="Q8" s="26" t="n"/>
+      <c r="Q8" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="R8" s="25" t="n"/>
       <c r="S8" s="24" t="n"/>
       <c r="T8" s="24" t="n"/>
@@ -7506,42 +7559,58 @@
         </is>
       </c>
       <c r="B9" s="28" t="n">
-        <v>235.31</v>
+        <v>237.13</v>
       </c>
       <c r="C9" s="29" t="n">
-        <v>23136</v>
+        <v>23429</v>
       </c>
       <c r="D9" s="29" t="n">
-        <v>104003</v>
+        <v>104539</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>2.262531</v>
+        <v>2.26834</v>
       </c>
       <c r="F9" s="29" t="n">
-        <v>4.495289</v>
+        <v>4.461949</v>
       </c>
       <c r="G9" s="29" t="n">
-        <v>4217</v>
+        <v>4237</v>
       </c>
       <c r="H9" s="28" t="n">
-        <v>0.0558</v>
+        <v>0.055966</v>
       </c>
       <c r="I9" s="30" t="n">
-        <v>4.054691</v>
-      </c>
-      <c r="J9" s="29" t="n"/>
-      <c r="K9" s="29" t="n"/>
-      <c r="L9" s="29" t="n"/>
-      <c r="M9" s="29" t="n"/>
-      <c r="N9" s="29" t="n"/>
-      <c r="O9" s="28" t="n"/>
-      <c r="P9" s="29" t="n"/>
-      <c r="Q9" s="30" t="n"/>
+        <v>4.053033</v>
+      </c>
+      <c r="J9" s="29" t="n">
+        <v>1633</v>
+      </c>
+      <c r="K9" s="29" t="n">
+        <v>2342</v>
+      </c>
+      <c r="L9" s="29" t="n">
+        <v>93</v>
+      </c>
+      <c r="M9" s="29" t="n">
+        <v>52</v>
+      </c>
+      <c r="N9" s="29" t="n">
+        <v>4</v>
+      </c>
+      <c r="O9" s="28" t="n">
+        <v>139.033715</v>
+      </c>
+      <c r="P9" s="29" t="n">
+        <v>0.5863185383544891</v>
+      </c>
+      <c r="Q9" s="30" t="n">
+        <v>0.1707941929974381</v>
+      </c>
       <c r="R9" s="29" t="n">
         <v>228</v>
       </c>
       <c r="S9" s="28" t="n">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="T9" s="28" t="n">
         <v>350.6</v>
@@ -7552,7 +7621,7 @@
         </is>
       </c>
       <c r="AA9" t="n">
-        <v>2980100</v>
+        <v>2997795</v>
       </c>
       <c r="AC9" t="inlineStr">
         <is>
@@ -7570,42 +7639,52 @@
         </is>
       </c>
       <c r="B10" s="24" t="n">
-        <v>61.53</v>
+        <v>64.09</v>
       </c>
       <c r="C10" s="25" t="n">
-        <v>17451</v>
+        <v>17874</v>
       </c>
       <c r="D10" s="25" t="n">
-        <v>35393</v>
+        <v>37099</v>
       </c>
       <c r="E10" s="24" t="n">
-        <v>1.738479</v>
+        <v>1.72754</v>
       </c>
       <c r="F10" s="25" t="n">
-        <v>2.028136</v>
+        <v>2.075585</v>
       </c>
       <c r="G10" s="25" t="n">
-        <v>1050</v>
+        <v>1098</v>
       </c>
       <c r="H10" s="24" t="n">
-        <v>0.0586</v>
+        <v>0.05837</v>
       </c>
       <c r="I10" s="26" t="n">
-        <v>2.966688</v>
-      </c>
-      <c r="J10" s="25" t="n"/>
-      <c r="K10" s="25" t="n"/>
-      <c r="L10" s="25" t="n"/>
-      <c r="M10" s="25" t="n"/>
+        <v>2.959649</v>
+      </c>
+      <c r="J10" s="25" t="n">
+        <v>408</v>
+      </c>
+      <c r="K10" s="25" t="n">
+        <v>440</v>
+      </c>
+      <c r="L10" s="25" t="n">
+        <v>42</v>
+      </c>
+      <c r="M10" s="25" t="n">
+        <v>6</v>
+      </c>
       <c r="N10" s="25" t="n"/>
       <c r="O10" s="24" t="n"/>
       <c r="P10" s="25" t="n"/>
-      <c r="Q10" s="26" t="n"/>
+      <c r="Q10" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="R10" s="25" t="n">
         <v>2</v>
       </c>
       <c r="S10" s="24" t="n">
-        <v>30.77</v>
+        <v>32.05</v>
       </c>
       <c r="T10" s="24" t="n">
         <v>72.47</v>
@@ -7616,7 +7695,7 @@
         </is>
       </c>
       <c r="AA10" t="n">
-        <v>688787</v>
+        <v>693603</v>
       </c>
       <c r="AC10" t="inlineStr">
         <is>
@@ -7634,42 +7713,58 @@
         </is>
       </c>
       <c r="B11" s="28" t="n">
-        <v>1141.96</v>
+        <v>1144.73</v>
       </c>
       <c r="C11" s="29" t="n">
         <v>211812</v>
       </c>
       <c r="D11" s="29" t="n">
-        <v>1117030</v>
+        <v>1119328</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>1.022318</v>
+        <v>1.022694</v>
       </c>
       <c r="F11" s="29" t="n">
-        <v>5.273686</v>
+        <v>5.284535</v>
       </c>
       <c r="G11" s="29" t="n">
-        <v>38724</v>
+        <v>38803</v>
       </c>
       <c r="H11" s="28" t="n">
-        <v>0.02949</v>
+        <v>0.029501</v>
       </c>
       <c r="I11" s="30" t="n">
-        <v>3.466693</v>
-      </c>
-      <c r="J11" s="29" t="n"/>
-      <c r="K11" s="29" t="n"/>
-      <c r="L11" s="29" t="n"/>
-      <c r="M11" s="29" t="n"/>
-      <c r="N11" s="29" t="n"/>
-      <c r="O11" s="28" t="n"/>
-      <c r="P11" s="29" t="n"/>
-      <c r="Q11" s="30" t="n"/>
+        <v>3.466634</v>
+      </c>
+      <c r="J11" s="29" t="n">
+        <v>7988</v>
+      </c>
+      <c r="K11" s="29" t="n">
+        <v>9380</v>
+      </c>
+      <c r="L11" s="29" t="n">
+        <v>204</v>
+      </c>
+      <c r="M11" s="29" t="n">
+        <v>39</v>
+      </c>
+      <c r="N11" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="O11" s="28" t="n">
+        <v>248.444281</v>
+      </c>
+      <c r="P11" s="29" t="n">
+        <v>0.2170330829103806</v>
+      </c>
+      <c r="Q11" s="30" t="n">
+        <v>0.06396588486140725</v>
+      </c>
       <c r="R11" s="29" t="n">
         <v>90</v>
       </c>
       <c r="S11" s="28" t="n">
-        <v>12.69</v>
+        <v>12.72</v>
       </c>
       <c r="T11" s="28" t="n">
         <v>49.67</v>
@@ -7744,31 +7839,47 @@
         </is>
       </c>
       <c r="B13" s="32" t="n">
-        <v>3010.41</v>
+        <v>3029.13</v>
       </c>
       <c r="C13" s="33" t="n"/>
       <c r="D13" s="33" t="n">
-        <v>688787</v>
+        <v>693603</v>
       </c>
       <c r="E13" s="32" t="n">
-        <v>4.370596425310001</v>
+        <v>4.367238896025537</v>
       </c>
       <c r="F13" s="33" t="n"/>
       <c r="G13" s="33" t="n">
-        <v>44020</v>
+        <v>44351</v>
       </c>
       <c r="H13" s="32" t="n">
-        <v>0.06838732394366197</v>
+        <v>0.06829902369732363</v>
       </c>
       <c r="I13" s="34" t="n"/>
-      <c r="J13" s="33" t="n"/>
-      <c r="K13" s="33" t="n"/>
-      <c r="L13" s="33" t="n"/>
-      <c r="M13" s="33" t="n"/>
-      <c r="N13" s="33" t="n"/>
-      <c r="O13" s="32" t="n"/>
-      <c r="P13" s="33" t="n"/>
-      <c r="Q13" s="34" t="n"/>
+      <c r="J13" s="33" t="n">
+        <v>31097</v>
+      </c>
+      <c r="K13" s="33" t="n">
+        <v>40050</v>
+      </c>
+      <c r="L13" s="33" t="n">
+        <v>3237</v>
+      </c>
+      <c r="M13" s="33" t="n">
+        <v>1363</v>
+      </c>
+      <c r="N13" s="33" t="n">
+        <v>185</v>
+      </c>
+      <c r="O13" s="32" t="n">
+        <v>9187.598484999999</v>
+      </c>
+      <c r="P13" s="33" t="n">
+        <v>3.033081605939659</v>
+      </c>
+      <c r="Q13" s="34" t="n">
+        <v>0.4619225967540574</v>
+      </c>
       <c r="R13" s="33" t="n"/>
       <c r="S13" s="32" t="n"/>
       <c r="T13" s="32" t="n"/>
@@ -7778,7 +7889,7 @@
         </is>
       </c>
       <c r="AA13" t="n">
-        <v>55131</v>
+        <v>55313</v>
       </c>
       <c r="AC13" t="inlineStr">
         <is>
@@ -7796,18 +7907,18 @@
         </is>
       </c>
       <c r="B14" s="24" t="n">
-        <v>453.98</v>
+        <v>455.36</v>
       </c>
       <c r="C14" s="25" t="n"/>
       <c r="D14" s="25" t="n">
-        <v>154176</v>
+        <v>154895</v>
       </c>
       <c r="E14" s="24" t="n">
         <v>2.94</v>
       </c>
       <c r="F14" s="25" t="n"/>
       <c r="G14" s="25" t="n">
-        <v>7376</v>
+        <v>7398</v>
       </c>
       <c r="H14" s="24" t="n">
         <v>0.06</v>
@@ -7815,14 +7926,30 @@
       <c r="I14" s="26" t="n">
         <v>4.78</v>
       </c>
-      <c r="J14" s="25" t="n"/>
-      <c r="K14" s="25" t="n"/>
-      <c r="L14" s="25" t="n"/>
-      <c r="M14" s="25" t="n"/>
-      <c r="N14" s="25" t="n"/>
-      <c r="O14" s="24" t="n"/>
-      <c r="P14" s="25" t="n"/>
-      <c r="Q14" s="26" t="n"/>
+      <c r="J14" s="25" t="n">
+        <v>4500</v>
+      </c>
+      <c r="K14" s="25" t="n">
+        <v>5605</v>
+      </c>
+      <c r="L14" s="25" t="n">
+        <v>435</v>
+      </c>
+      <c r="M14" s="25" t="n">
+        <v>172</v>
+      </c>
+      <c r="N14" s="25" t="n">
+        <v>29</v>
+      </c>
+      <c r="O14" s="24" t="n">
+        <v>1290.379205</v>
+      </c>
+      <c r="P14" s="25" t="n">
+        <v>2.833756159961349</v>
+      </c>
+      <c r="Q14" s="26" t="n">
+        <v>0.5173951828724354</v>
+      </c>
       <c r="R14" s="25" t="n"/>
       <c r="S14" s="24" t="n"/>
       <c r="T14" s="24" t="n"/>
@@ -7832,7 +7959,7 @@
         </is>
       </c>
       <c r="AA14" t="n">
-        <v>44020</v>
+        <v>44351</v>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
@@ -7850,18 +7977,18 @@
         </is>
       </c>
       <c r="B15" s="28" t="n">
-        <v>1258.98</v>
+        <v>1266.48</v>
       </c>
       <c r="C15" s="29" t="n"/>
       <c r="D15" s="29" t="n">
-        <v>57840</v>
+        <v>58313</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>21.77</v>
+        <v>21.72</v>
       </c>
       <c r="F15" s="29" t="n"/>
       <c r="G15" s="29" t="n">
-        <v>19430</v>
+        <v>19589</v>
       </c>
       <c r="H15" s="28" t="n">
         <v>0.06</v>
@@ -7869,14 +7996,30 @@
       <c r="I15" s="30" t="n">
         <v>33.59</v>
       </c>
-      <c r="J15" s="29" t="n"/>
-      <c r="K15" s="29" t="n"/>
-      <c r="L15" s="29" t="n"/>
-      <c r="M15" s="29" t="n"/>
-      <c r="N15" s="29" t="n"/>
-      <c r="O15" s="28" t="n"/>
-      <c r="P15" s="29" t="n"/>
-      <c r="Q15" s="30" t="n"/>
+      <c r="J15" s="29" t="n">
+        <v>14387</v>
+      </c>
+      <c r="K15" s="29" t="n">
+        <v>19522</v>
+      </c>
+      <c r="L15" s="29" t="n">
+        <v>2069</v>
+      </c>
+      <c r="M15" s="29" t="n">
+        <v>800</v>
+      </c>
+      <c r="N15" s="29" t="n">
+        <v>111</v>
+      </c>
+      <c r="O15" s="28" t="n">
+        <v>5953.989020999999</v>
+      </c>
+      <c r="P15" s="29" t="n">
+        <v>4.701210458120143</v>
+      </c>
+      <c r="Q15" s="30" t="n">
+        <v>0.5685892838848479</v>
+      </c>
       <c r="R15" s="29" t="n"/>
       <c r="S15" s="28" t="n"/>
       <c r="T15" s="28" t="n"/>
@@ -7888,18 +8031,18 @@
         </is>
       </c>
       <c r="B16" s="24" t="n">
-        <v>242.62</v>
+        <v>242.91</v>
       </c>
       <c r="C16" s="25" t="n"/>
       <c r="D16" s="25" t="n">
-        <v>53513</v>
+        <v>53552</v>
       </c>
       <c r="E16" s="24" t="n">
-        <v>4.53</v>
+        <v>4.54</v>
       </c>
       <c r="F16" s="25" t="n"/>
       <c r="G16" s="25" t="n">
-        <v>1926</v>
+        <v>1930</v>
       </c>
       <c r="H16" s="24" t="n">
         <v>0.13</v>
@@ -7907,14 +8050,24 @@
       <c r="I16" s="26" t="n">
         <v>3.6</v>
       </c>
-      <c r="J16" s="25" t="n"/>
-      <c r="K16" s="25" t="n"/>
-      <c r="L16" s="25" t="n"/>
-      <c r="M16" s="25" t="n"/>
+      <c r="J16" s="25" t="n">
+        <v>1358</v>
+      </c>
+      <c r="K16" s="25" t="n">
+        <v>1576</v>
+      </c>
+      <c r="L16" s="25" t="n">
+        <v>46</v>
+      </c>
+      <c r="M16" s="25" t="n">
+        <v>19</v>
+      </c>
       <c r="N16" s="25" t="n"/>
       <c r="O16" s="24" t="n"/>
       <c r="P16" s="25" t="n"/>
-      <c r="Q16" s="26" t="n"/>
+      <c r="Q16" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="R16" s="25" t="n"/>
       <c r="S16" s="24" t="n"/>
       <c r="T16" s="24" t="n"/>
@@ -7946,33 +8099,49 @@
         </is>
       </c>
       <c r="B17" s="28" t="n">
-        <v>227.4</v>
+        <v>228.21</v>
       </c>
       <c r="C17" s="29" t="n"/>
       <c r="D17" s="29" t="n">
-        <v>16690</v>
+        <v>16741</v>
       </c>
       <c r="E17" s="28" t="n">
         <v>13.63</v>
       </c>
       <c r="F17" s="29" t="n"/>
       <c r="G17" s="29" t="n">
-        <v>1115</v>
+        <v>1121</v>
       </c>
       <c r="H17" s="28" t="n">
         <v>0.2</v>
       </c>
       <c r="I17" s="30" t="n">
-        <v>6.68</v>
-      </c>
-      <c r="J17" s="29" t="n"/>
-      <c r="K17" s="29" t="n"/>
-      <c r="L17" s="29" t="n"/>
-      <c r="M17" s="29" t="n"/>
-      <c r="N17" s="29" t="n"/>
-      <c r="O17" s="28" t="n"/>
-      <c r="P17" s="29" t="n"/>
-      <c r="Q17" s="30" t="n"/>
+        <v>6.7</v>
+      </c>
+      <c r="J17" s="29" t="n">
+        <v>781</v>
+      </c>
+      <c r="K17" s="29" t="n">
+        <v>974</v>
+      </c>
+      <c r="L17" s="29" t="n">
+        <v>58</v>
+      </c>
+      <c r="M17" s="29" t="n">
+        <v>31</v>
+      </c>
+      <c r="N17" s="29" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" s="28" t="n">
+        <v>115.698619</v>
+      </c>
+      <c r="P17" s="29" t="n">
+        <v>0.5069831251917094</v>
+      </c>
+      <c r="Q17" s="30" t="n">
+        <v>0.3080082135523614</v>
+      </c>
       <c r="R17" s="29" t="n"/>
       <c r="S17" s="28" t="n"/>
       <c r="T17" s="28" t="n"/>
@@ -7982,7 +8151,7 @@
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>0</v>
+        <v>12684</v>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
@@ -7990,7 +8159,7 @@
         </is>
       </c>
       <c r="AD17" s="12" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="18">
@@ -8000,33 +8169,43 @@
         </is>
       </c>
       <c r="B18" s="24" t="n">
-        <v>114.85</v>
+        <v>115.53</v>
       </c>
       <c r="C18" s="25" t="n"/>
       <c r="D18" s="25" t="n">
-        <v>13492</v>
+        <v>13606</v>
       </c>
       <c r="E18" s="24" t="n">
-        <v>8.51</v>
+        <v>8.49</v>
       </c>
       <c r="F18" s="25" t="n"/>
       <c r="G18" s="25" t="n">
-        <v>871</v>
+        <v>878</v>
       </c>
       <c r="H18" s="24" t="n">
         <v>0.13</v>
       </c>
       <c r="I18" s="26" t="n">
-        <v>6.46</v>
-      </c>
-      <c r="J18" s="25" t="n"/>
-      <c r="K18" s="25" t="n"/>
-      <c r="L18" s="25" t="n"/>
-      <c r="M18" s="25" t="n"/>
+        <v>6.45</v>
+      </c>
+      <c r="J18" s="25" t="n">
+        <v>683</v>
+      </c>
+      <c r="K18" s="25" t="n">
+        <v>767</v>
+      </c>
+      <c r="L18" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="M18" s="25" t="n">
+        <v>3</v>
+      </c>
       <c r="N18" s="25" t="n"/>
       <c r="O18" s="24" t="n"/>
       <c r="P18" s="25" t="n"/>
-      <c r="Q18" s="26" t="n"/>
+      <c r="Q18" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="R18" s="25" t="n"/>
       <c r="S18" s="24" t="n"/>
       <c r="T18" s="24" t="n"/>
@@ -8036,7 +8215,7 @@
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>0</v>
+        <v>40050</v>
       </c>
       <c r="AC18" t="inlineStr">
         <is>
@@ -8044,7 +8223,7 @@
         </is>
       </c>
       <c r="AD18" s="12" t="n">
-        <v>0</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="19">
@@ -8054,33 +8233,49 @@
         </is>
       </c>
       <c r="B19" s="28" t="n">
-        <v>56.16</v>
+        <v>56.9</v>
       </c>
       <c r="C19" s="29" t="n"/>
       <c r="D19" s="29" t="n">
-        <v>7520</v>
+        <v>7577</v>
       </c>
       <c r="E19" s="28" t="n">
-        <v>7.47</v>
+        <v>7.51</v>
       </c>
       <c r="F19" s="29" t="n"/>
       <c r="G19" s="29" t="n">
-        <v>652</v>
+        <v>661</v>
       </c>
       <c r="H19" s="28" t="n">
         <v>0.09</v>
       </c>
       <c r="I19" s="30" t="n">
-        <v>8.67</v>
-      </c>
-      <c r="J19" s="29" t="n"/>
-      <c r="K19" s="29" t="n"/>
-      <c r="L19" s="29" t="n"/>
-      <c r="M19" s="29" t="n"/>
-      <c r="N19" s="29" t="n"/>
-      <c r="O19" s="28" t="n"/>
-      <c r="P19" s="29" t="n"/>
-      <c r="Q19" s="30" t="n"/>
+        <v>8.720000000000001</v>
+      </c>
+      <c r="J19" s="29" t="n">
+        <v>432</v>
+      </c>
+      <c r="K19" s="29" t="n">
+        <v>513</v>
+      </c>
+      <c r="L19" s="29" t="n">
+        <v>55</v>
+      </c>
+      <c r="M19" s="29" t="n">
+        <v>7</v>
+      </c>
+      <c r="N19" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" s="28" t="n">
+        <v>19.537635</v>
+      </c>
+      <c r="P19" s="29" t="n">
+        <v>0.3433679261862917</v>
+      </c>
+      <c r="Q19" s="30" t="n">
+        <v>0.1949317738791423</v>
+      </c>
       <c r="R19" s="29" t="n"/>
       <c r="S19" s="28" t="n"/>
       <c r="T19" s="28" t="n"/>
@@ -8092,33 +8287,43 @@
         </is>
       </c>
       <c r="B20" s="24" t="n">
-        <v>53.91</v>
+        <v>55.1</v>
       </c>
       <c r="C20" s="25" t="n"/>
       <c r="D20" s="25" t="n">
-        <v>15255</v>
+        <v>15351</v>
       </c>
       <c r="E20" s="24" t="n">
-        <v>3.53</v>
+        <v>3.59</v>
       </c>
       <c r="F20" s="25" t="n"/>
       <c r="G20" s="25" t="n">
-        <v>561</v>
+        <v>571</v>
       </c>
       <c r="H20" s="24" t="n">
         <v>0.1</v>
       </c>
       <c r="I20" s="26" t="n">
-        <v>3.68</v>
-      </c>
-      <c r="J20" s="25" t="n"/>
-      <c r="K20" s="25" t="n"/>
-      <c r="L20" s="25" t="n"/>
-      <c r="M20" s="25" t="n"/>
+        <v>3.72</v>
+      </c>
+      <c r="J20" s="25" t="n">
+        <v>348</v>
+      </c>
+      <c r="K20" s="25" t="n">
+        <v>396</v>
+      </c>
+      <c r="L20" s="25" t="n">
+        <v>17</v>
+      </c>
+      <c r="M20" s="25" t="n">
+        <v>1</v>
+      </c>
       <c r="N20" s="25" t="n"/>
       <c r="O20" s="24" t="n"/>
       <c r="P20" s="25" t="n"/>
-      <c r="Q20" s="26" t="n"/>
+      <c r="Q20" s="26" t="n">
+        <v>0</v>
+      </c>
       <c r="R20" s="25" t="n"/>
       <c r="S20" s="24" t="n"/>
       <c r="T20" s="24" t="n"/>
@@ -8150,33 +8355,49 @@
         </is>
       </c>
       <c r="B21" s="28" t="n">
-        <v>602.51</v>
+        <v>608.64</v>
       </c>
       <c r="C21" s="29" t="n"/>
       <c r="D21" s="29" t="n">
-        <v>370301</v>
+        <v>373568</v>
       </c>
       <c r="E21" s="28" t="n">
         <v>1.63</v>
       </c>
       <c r="F21" s="29" t="n"/>
       <c r="G21" s="29" t="n">
-        <v>12089</v>
+        <v>12203</v>
       </c>
       <c r="H21" s="28" t="n">
         <v>0.05</v>
       </c>
       <c r="I21" s="30" t="n">
-        <v>3.26</v>
-      </c>
-      <c r="J21" s="29" t="n"/>
-      <c r="K21" s="29" t="n"/>
-      <c r="L21" s="29" t="n"/>
-      <c r="M21" s="29" t="n"/>
-      <c r="N21" s="29" t="n"/>
-      <c r="O21" s="28" t="n"/>
-      <c r="P21" s="29" t="n"/>
-      <c r="Q21" s="30" t="n"/>
+        <v>3.27</v>
+      </c>
+      <c r="J21" s="29" t="n">
+        <v>8608</v>
+      </c>
+      <c r="K21" s="29" t="n">
+        <v>10697</v>
+      </c>
+      <c r="L21" s="29" t="n">
+        <v>537</v>
+      </c>
+      <c r="M21" s="29" t="n">
+        <v>330</v>
+      </c>
+      <c r="N21" s="29" t="n">
+        <v>41</v>
+      </c>
+      <c r="O21" s="28" t="n">
+        <v>1807.994005</v>
+      </c>
+      <c r="P21" s="29" t="n">
+        <v>2.970547458267613</v>
+      </c>
+      <c r="Q21" s="30" t="n">
+        <v>0.3832850331868748</v>
+      </c>
       <c r="R21" s="29" t="n"/>
       <c r="S21" s="28" t="n"/>
       <c r="T21" s="28" t="n"/>
@@ -8186,7 +8407,7 @@
         </is>
       </c>
       <c r="AA21" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AC21" t="inlineStr">
         <is>
@@ -8194,7 +8415,7 @@
         </is>
       </c>
       <c r="AD21" s="12" t="n">
-        <v>0</v>
+        <v>195.11</v>
       </c>
     </row>
     <row r="22">
@@ -8204,7 +8425,7 @@
         </is>
       </c>
       <c r="AA22" t="n">
-        <v>0</v>
+        <v>185</v>
       </c>
       <c r="AC22" t="inlineStr">
         <is>
@@ -8212,7 +8433,7 @@
         </is>
       </c>
       <c r="AD22" s="12" t="n">
-        <v>0</v>
+        <v>16.37</v>
       </c>
     </row>
     <row r="24">
@@ -8234,7 +8455,7 @@
         </is>
       </c>
       <c r="AA25" s="12" t="n">
-        <v>0</v>
+        <v>387.477996</v>
       </c>
     </row>
     <row r="26">
@@ -8244,7 +8465,7 @@
         </is>
       </c>
       <c r="AA26" s="12" t="n">
-        <v>0</v>
+        <v>9187.598484999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>